<commit_message>
Source excel files upload
</commit_message>
<xml_diff>
--- a/_sources/LogicalModelExample_v2.xlsx
+++ b/_sources/LogicalModelExample_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hl7europe-my.sharepoint.com/personal/roberta_hl7europe_org/Documents/Roberta/IDEA4RC/Cancer Model/LogicalModel/Esempi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="123" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4CA70DA7-489E-4399-80D9-ABE6F5DD5EE1}"/>
+  <xr:revisionPtr revIDLastSave="140" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1752DA9-9DA2-4C5D-83FC-FAD929245D67}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -293,21 +293,6 @@
     <t>Surgery/1</t>
   </si>
   <si>
-    <t>stageComponent1</t>
-  </si>
-  <si>
-    <t>stageComponent2</t>
-  </si>
-  <si>
-    <t>stageComponent3</t>
-  </si>
-  <si>
-    <t>code</t>
-  </si>
-  <si>
-    <t>value</t>
-  </si>
-  <si>
     <t>Text: TNM</t>
   </si>
   <si>
@@ -330,6 +315,21 @@
   </si>
   <si>
     <t>Text: N1</t>
+  </si>
+  <si>
+    <t>Value1</t>
+  </si>
+  <si>
+    <t>Value2</t>
+  </si>
+  <si>
+    <t>Value3</t>
+  </si>
+  <si>
+    <t>Code</t>
+  </si>
+  <si>
+    <t>Value</t>
   </si>
 </sst>
 </file>
@@ -458,7 +458,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="40">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
@@ -481,78 +481,57 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="right"/>
-    </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normale" xfId="0" builtinId="0"/>
@@ -836,468 +815,471 @@
   <dimension ref="A1:W12"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="32.140625" style="14" customWidth="1"/>
-    <col min="2" max="2" width="28.42578125" style="14" customWidth="1"/>
-    <col min="3" max="3" width="9.140625" style="14"/>
-    <col min="4" max="4" width="30.7109375" style="14" customWidth="1"/>
-    <col min="5" max="5" width="9.140625" style="14"/>
-    <col min="6" max="7" width="8.85546875" style="14"/>
-    <col min="8" max="8" width="13" style="14" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" style="14"/>
-    <col min="10" max="10" width="24.140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="24.140625" style="14" customWidth="1"/>
-    <col min="12" max="12" width="10.85546875" style="14" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="9.140625" style="14"/>
-    <col min="14" max="14" width="29.28515625" style="14" customWidth="1"/>
-    <col min="15" max="15" width="13.7109375" style="14" customWidth="1"/>
-    <col min="16" max="16" width="9.140625" style="14"/>
-    <col min="17" max="18" width="23.140625" style="35" customWidth="1"/>
-    <col min="19" max="19" width="15" style="35" customWidth="1"/>
-    <col min="20" max="20" width="11.42578125" style="14" customWidth="1"/>
-    <col min="21" max="21" width="9.140625" style="14"/>
-    <col min="22" max="22" width="36.140625" style="14" bestFit="1" customWidth="1"/>
-    <col min="23" max="23" width="22.7109375" style="14" bestFit="1" customWidth="1"/>
-    <col min="24" max="16384" width="9.140625" style="14"/>
+    <col min="1" max="1" width="32.140625" customWidth="1"/>
+    <col min="2" max="2" width="28.42578125" customWidth="1"/>
+    <col min="4" max="4" width="30.7109375" customWidth="1"/>
+    <col min="6" max="7" width="8.85546875"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="10" max="10" width="24.140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="24.140625" customWidth="1"/>
+    <col min="12" max="12" width="10.85546875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="29.28515625" customWidth="1"/>
+    <col min="15" max="15" width="13.7109375" customWidth="1"/>
+    <col min="17" max="18" width="23.140625" style="21" customWidth="1"/>
+    <col min="19" max="19" width="15" style="21" customWidth="1"/>
+    <col min="20" max="20" width="11.42578125" customWidth="1"/>
+    <col min="22" max="22" width="36.140625" bestFit="1" customWidth="1"/>
+    <col min="23" max="23" width="22.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="23" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="13"/>
-      <c r="D1" s="13" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="13"/>
-      <c r="F1" s="15"/>
-      <c r="G1" s="13" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="13"/>
-      <c r="J1" s="13" t="s">
+      <c r="E1" s="23"/>
+      <c r="F1" s="12"/>
+      <c r="G1" s="23" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="23"/>
+      <c r="J1" s="23" t="s">
         <v>57</v>
       </c>
-      <c r="K1" s="13"/>
-      <c r="L1" s="13"/>
-      <c r="M1" s="15"/>
-      <c r="N1" s="13" t="s">
+      <c r="K1" s="23"/>
+      <c r="L1" s="23"/>
+      <c r="M1" s="12"/>
+      <c r="N1" s="23" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="13"/>
-      <c r="Q1" s="16" t="s">
+      <c r="O1" s="23"/>
+      <c r="Q1" s="24" t="s">
         <v>57</v>
       </c>
-      <c r="R1" s="16"/>
-      <c r="S1" s="16"/>
-      <c r="T1" s="15"/>
-      <c r="V1" s="13" t="s">
+      <c r="R1" s="24"/>
+      <c r="S1" s="24"/>
+      <c r="T1" s="12"/>
+      <c r="V1" s="23" t="s">
         <v>67</v>
       </c>
-      <c r="W1" s="13"/>
+      <c r="W1" s="23"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="18">
+      <c r="B2" s="1">
         <v>11</v>
       </c>
-      <c r="D2" s="17" t="s">
+      <c r="D2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="E2" s="19">
-        <v>1</v>
-      </c>
-      <c r="G2" s="19" t="s">
+      <c r="E2" s="2">
+        <v>1</v>
+      </c>
+      <c r="G2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="H2" s="19">
-        <v>1</v>
-      </c>
-      <c r="J2" s="20" t="s">
+      <c r="H2" s="2">
+        <v>1</v>
+      </c>
+      <c r="J2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="21"/>
-      <c r="L2" s="19">
-        <v>1</v>
-      </c>
-      <c r="N2" s="19" t="s">
+      <c r="K2" s="26"/>
+      <c r="L2" s="2">
+        <v>1</v>
+      </c>
+      <c r="N2" s="2" t="s">
         <v>0</v>
       </c>
-      <c r="O2" s="19">
-        <v>1</v>
-      </c>
-      <c r="Q2" s="20" t="s">
+      <c r="O2" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="25" t="s">
         <v>0</v>
       </c>
-      <c r="R2" s="21"/>
-      <c r="S2" s="22">
+      <c r="R2" s="26"/>
+      <c r="S2" s="6">
         <v>2</v>
       </c>
-      <c r="V2" s="17" t="s">
+      <c r="V2" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="W2" s="19">
+      <c r="W2" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:23" ht="135" x14ac:dyDescent="0.25">
-      <c r="A3" s="23" t="s">
+      <c r="A3" s="8" t="s">
         <v>56</v>
       </c>
-      <c r="B3" s="19">
+      <c r="B3" s="2">
         <v>22</v>
       </c>
-      <c r="D3" s="23" t="s">
+      <c r="D3" s="8" t="s">
         <v>4</v>
       </c>
-      <c r="E3" s="19">
+      <c r="E3" s="2">
         <v>1975</v>
       </c>
-      <c r="G3" s="24" t="s">
+      <c r="G3" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="H3" s="25" t="s">
+      <c r="H3" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="J3" s="26" t="s">
+      <c r="J3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="K3" s="26"/>
-      <c r="L3" s="19">
-        <v>1</v>
-      </c>
-      <c r="N3" s="24" t="s">
+      <c r="K3" s="14"/>
+      <c r="L3" s="2">
+        <v>1</v>
+      </c>
+      <c r="N3" s="7" t="s">
         <v>56</v>
       </c>
-      <c r="O3" s="19">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="26" t="s">
+      <c r="O3" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="14" t="s">
         <v>54</v>
       </c>
-      <c r="R3" s="26"/>
-      <c r="S3" s="22">
-        <v>1</v>
-      </c>
-      <c r="V3" s="19" t="s">
+      <c r="R3" s="14"/>
+      <c r="S3" s="6">
+        <v>1</v>
+      </c>
+      <c r="V3" s="2" t="s">
         <v>56</v>
       </c>
-      <c r="W3" s="19">
+      <c r="W3" s="2">
         <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:23" ht="105" x14ac:dyDescent="0.25">
-      <c r="A4" s="27" t="s">
+      <c r="A4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="B4" s="25" t="s">
+      <c r="B4" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="D4" s="28" t="s">
+      <c r="D4" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="E4" s="29" t="s">
+      <c r="E4" s="16" t="s">
         <v>6</v>
       </c>
-      <c r="F4" s="30"/>
-      <c r="G4" s="24" t="s">
+      <c r="F4" s="17"/>
+      <c r="G4" s="7" t="s">
         <v>3</v>
       </c>
-      <c r="H4" s="25" t="s">
+      <c r="H4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="20" t="s">
+      <c r="J4" s="25" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="21"/>
-      <c r="L4" s="31" t="s">
+      <c r="K4" s="26"/>
+      <c r="L4" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="N4" s="14" t="s">
+        <v>54</v>
+      </c>
+      <c r="O4" s="2">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="R4" s="26"/>
+      <c r="S4" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>54</v>
+      </c>
+      <c r="W4" s="2">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:23" ht="75" x14ac:dyDescent="0.25">
+      <c r="A5" s="15" t="s">
+        <v>3</v>
+      </c>
+      <c r="B5" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="19"/>
+      <c r="G5" s="19"/>
+      <c r="H5" s="19"/>
+      <c r="J5" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="K5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L5" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="M5" s="20"/>
+      <c r="N5" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="O5" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="Q5" s="27" t="s">
+        <v>83</v>
+      </c>
+      <c r="R5" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S5" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="T5" s="20"/>
+      <c r="V5" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="W5" s="2" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" ht="30" x14ac:dyDescent="0.25">
+      <c r="A6" s="15" t="s">
+        <v>64</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>5</v>
+      </c>
+      <c r="E6" s="6" t="s">
+        <v>16</v>
+      </c>
+      <c r="F6" s="21"/>
+      <c r="G6" s="21"/>
+      <c r="H6" s="21"/>
+      <c r="J6" s="28"/>
+      <c r="K6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="N6" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="Q6" s="28"/>
+      <c r="R6" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="S6" s="6" t="s">
+        <v>79</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="W6" s="2" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" ht="30" x14ac:dyDescent="0.25">
+      <c r="A7" s="9" t="s">
+        <v>8</v>
+      </c>
+      <c r="B7" s="22" t="s">
+        <v>13</v>
+      </c>
+      <c r="J7" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="K7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="N7" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="O7" s="4">
+        <v>43263</v>
+      </c>
+      <c r="Q7" s="27" t="s">
+        <v>84</v>
+      </c>
+      <c r="R7" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S7" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="W7" s="4">
+        <v>43353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:23" ht="105" x14ac:dyDescent="0.25">
+      <c r="A8" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="B8" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J8" s="28"/>
+      <c r="K8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L8" s="6" t="s">
         <v>80</v>
       </c>
-      <c r="N4" s="26" t="s">
-        <v>54</v>
-      </c>
-      <c r="O4" s="19">
-        <v>1</v>
-      </c>
-      <c r="Q4" s="20" t="s">
-        <v>17</v>
-      </c>
-      <c r="R4" s="21"/>
-      <c r="S4" s="31" t="s">
-        <v>80</v>
-      </c>
-      <c r="V4" s="19" t="s">
-        <v>54</v>
-      </c>
-      <c r="W4" s="19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:23" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="27" t="s">
+      <c r="N8" s="14" t="s">
         <v>3</v>
       </c>
-      <c r="B5" s="25" t="s">
+      <c r="O8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="D5" s="28" t="s">
-        <v>15</v>
-      </c>
-      <c r="E5" s="28" t="s">
-        <v>16</v>
-      </c>
-      <c r="F5" s="32"/>
-      <c r="G5" s="32"/>
-      <c r="H5" s="32"/>
-      <c r="J5" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="K5" s="22" t="s">
+      <c r="Q8" s="28"/>
+      <c r="R8" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="S8" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="W8" s="4">
+        <v>43385</v>
+      </c>
+    </row>
+    <row r="9" spans="1:23" ht="75" x14ac:dyDescent="0.25">
+      <c r="A9" s="8" t="s">
+        <v>10</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J9" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="K9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="L9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="L5" s="31" t="s">
+      <c r="Q9" s="27" t="s">
+        <v>85</v>
+      </c>
+      <c r="R9" s="6" t="s">
+        <v>86</v>
+      </c>
+      <c r="S9" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>3</v>
+      </c>
+      <c r="W9" s="3" t="s">
+        <v>52</v>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" s="8" t="s">
+        <v>11</v>
+      </c>
+      <c r="B10" s="4">
+        <v>43221</v>
+      </c>
+      <c r="J10" s="28"/>
+      <c r="K10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="L10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="M5" s="34"/>
-      <c r="N5" s="26" t="s">
-        <v>58</v>
-      </c>
-      <c r="O5" s="25" t="s">
-        <v>16</v>
-      </c>
-      <c r="Q5" s="33" t="s">
-        <v>75</v>
-      </c>
-      <c r="R5" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="S5" s="31" t="s">
+      <c r="Q10" s="28"/>
+      <c r="R10" s="6" t="s">
+        <v>87</v>
+      </c>
+      <c r="S10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="T5" s="34"/>
-      <c r="V5" s="19" t="s">
-        <v>58</v>
-      </c>
-      <c r="W5" s="19" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="6" spans="1:23" ht="30" x14ac:dyDescent="0.25">
-      <c r="A6" s="27" t="s">
-        <v>64</v>
-      </c>
-      <c r="B6" s="25" t="s">
-        <v>59</v>
-      </c>
-      <c r="D6" s="28" t="s">
-        <v>5</v>
-      </c>
-      <c r="E6" s="22" t="s">
-        <v>16</v>
-      </c>
-      <c r="F6" s="35"/>
-      <c r="G6" s="35"/>
-      <c r="H6" s="35"/>
-      <c r="J6" s="36"/>
-      <c r="K6" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="L6" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="N6" s="26" t="s">
-        <v>21</v>
-      </c>
-      <c r="O6" s="19" t="s">
-        <v>24</v>
-      </c>
-      <c r="Q6" s="36"/>
-      <c r="R6" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="S6" s="22" t="s">
-        <v>84</v>
-      </c>
-      <c r="V6" s="19" t="s">
-        <v>21</v>
-      </c>
-      <c r="W6" s="19" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="7" spans="1:23" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="37" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" s="38" t="s">
-        <v>13</v>
-      </c>
-      <c r="J7" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="K7" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="L7" s="31" t="s">
-        <v>82</v>
-      </c>
-      <c r="N7" s="26" t="s">
-        <v>22</v>
-      </c>
-      <c r="O7" s="39">
-        <v>43263</v>
-      </c>
-      <c r="Q7" s="33" t="s">
-        <v>76</v>
-      </c>
-      <c r="R7" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="S7" s="31" t="s">
-        <v>82</v>
-      </c>
-      <c r="V7" s="19" t="s">
-        <v>45</v>
-      </c>
-      <c r="W7" s="39">
-        <v>43353</v>
-      </c>
-    </row>
-    <row r="8" spans="1:23" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" s="23" t="s">
-        <v>9</v>
-      </c>
-      <c r="B8" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J8" s="36"/>
-      <c r="K8" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="L8" s="22" t="s">
-        <v>85</v>
-      </c>
-      <c r="N8" s="26" t="s">
-        <v>3</v>
-      </c>
-      <c r="O8" s="25" t="s">
-        <v>52</v>
-      </c>
-      <c r="Q8" s="36"/>
-      <c r="R8" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="S8" s="22" t="s">
-        <v>87</v>
-      </c>
-      <c r="V8" s="19" t="s">
-        <v>46</v>
-      </c>
-      <c r="W8" s="39">
-        <v>43385</v>
-      </c>
-    </row>
-    <row r="9" spans="1:23" ht="75" x14ac:dyDescent="0.25">
-      <c r="A9" s="23" t="s">
-        <v>10</v>
-      </c>
-      <c r="B9" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J9" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="K9" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="L9" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="Q9" s="33" t="s">
-        <v>77</v>
-      </c>
-      <c r="R9" s="22" t="s">
-        <v>78</v>
-      </c>
-      <c r="S9" s="31" t="s">
-        <v>83</v>
-      </c>
-      <c r="V9" s="19" t="s">
-        <v>3</v>
-      </c>
-      <c r="W9" s="25" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A10" s="23" t="s">
-        <v>11</v>
-      </c>
-      <c r="B10" s="39">
-        <v>43221</v>
-      </c>
-      <c r="J10" s="36"/>
-      <c r="K10" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="L10" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="Q10" s="36"/>
-      <c r="R10" s="22" t="s">
-        <v>79</v>
-      </c>
-      <c r="S10" s="22" t="s">
-        <v>86</v>
-      </c>
-      <c r="V10" s="19" t="s">
+      <c r="V10" s="2" t="s">
         <v>68</v>
       </c>
-      <c r="W10" s="19" t="s">
+      <c r="W10" s="2" t="s">
         <v>69</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A11" s="19" t="s">
+      <c r="A11" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="B11" s="19" t="s">
-        <v>16</v>
-      </c>
-      <c r="J11" s="19" t="s">
+      <c r="B11" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="J11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="K11" s="19"/>
-      <c r="L11" s="19" t="s">
+      <c r="K11" s="2"/>
+      <c r="L11" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="Q11" s="22" t="s">
+      <c r="Q11" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="R11" s="22"/>
-      <c r="S11" s="22" t="s">
+      <c r="R11" s="6"/>
+      <c r="S11" s="6" t="s">
         <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="J12" s="19" t="s">
+      <c r="J12" s="2" t="s">
         <v>66</v>
       </c>
-      <c r="K12" s="19"/>
-      <c r="L12" s="19" t="s">
+      <c r="K12" s="2"/>
+      <c r="L12" s="2" t="s">
         <v>73</v>
       </c>
-      <c r="Q12" s="22" t="s">
+      <c r="Q12" s="6" t="s">
         <v>66</v>
       </c>
-      <c r="R12" s="22"/>
-      <c r="S12" s="22" t="s">
+      <c r="R12" s="6"/>
+      <c r="S12" s="6" t="s">
         <v>74</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="Q9:Q10"/>
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
@@ -1305,16 +1287,6 @@
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="N1:O1"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="Q9:Q10"/>
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1335,18 +1307,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="G1" s="12" t="s">
+      <c r="E1" s="23"/>
+      <c r="G1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="12"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1514,14 +1486,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="12"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1658,14 +1630,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="12"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1802,14 +1774,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="12"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1944,10 +1916,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="23"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2053,18 +2025,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="12"/>
-      <c r="G1" s="12" t="s">
+      <c r="E1" s="23"/>
+      <c r="G1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="12"/>
+      <c r="H1" s="23"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2232,14 +2204,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="12"/>
-      <c r="D1" s="12" t="s">
+      <c r="B1" s="23"/>
+      <c r="D1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="12"/>
+      <c r="E1" s="23"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2374,10 +2346,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="23" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="12"/>
+      <c r="B1" s="23"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">

</xml_diff>

<commit_message>
CancerStage Logical Model Update
</commit_message>
<xml_diff>
--- a/_sources/LogicalModelExample_v2.xlsx
+++ b/_sources/LogicalModelExample_v2.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://hl7europe-my.sharepoint.com/personal/roberta_hl7europe_org/Documents/Roberta/IDEA4RC/Cancer Model/LogicalModel/Esempi/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="140" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1752DA9-9DA2-4C5D-83FC-FAD929245D67}"/>
+  <xr:revisionPtr revIDLastSave="148" documentId="8_{ED9382E8-2342-4AE0-AA39-3164F895D6A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EB986FEE-57D3-4F37-B815-09EB38FA762D}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -317,19 +317,19 @@
     <t>Text: N1</t>
   </si>
   <si>
-    <t>Value1</t>
-  </si>
-  <si>
-    <t>Value2</t>
-  </si>
-  <si>
-    <t>Value3</t>
-  </si>
-  <si>
     <t>Code</t>
   </si>
   <si>
     <t>Value</t>
+  </si>
+  <si>
+    <t>StageValue1</t>
+  </si>
+  <si>
+    <t>StageValue2</t>
+  </si>
+  <si>
+    <t>StageValue3</t>
   </si>
 </sst>
 </file>
@@ -514,12 +514,6 @@
     <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -531,6 +525,12 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -833,39 +833,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:23" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>53</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>55</v>
       </c>
-      <c r="E1" s="23"/>
+      <c r="E1" s="27"/>
       <c r="F1" s="12"/>
-      <c r="G1" s="23" t="s">
-        <v>1</v>
-      </c>
-      <c r="H1" s="23"/>
-      <c r="J1" s="23" t="s">
+      <c r="G1" s="27" t="s">
+        <v>1</v>
+      </c>
+      <c r="H1" s="27"/>
+      <c r="J1" s="27" t="s">
         <v>57</v>
       </c>
-      <c r="K1" s="23"/>
-      <c r="L1" s="23"/>
+      <c r="K1" s="27"/>
+      <c r="L1" s="27"/>
       <c r="M1" s="12"/>
-      <c r="N1" s="23" t="s">
+      <c r="N1" s="27" t="s">
         <v>23</v>
       </c>
-      <c r="O1" s="23"/>
-      <c r="Q1" s="24" t="s">
+      <c r="O1" s="27"/>
+      <c r="Q1" s="28" t="s">
         <v>57</v>
       </c>
-      <c r="R1" s="24"/>
-      <c r="S1" s="24"/>
+      <c r="R1" s="28"/>
+      <c r="S1" s="28"/>
       <c r="T1" s="12"/>
-      <c r="V1" s="23" t="s">
+      <c r="V1" s="27" t="s">
         <v>67</v>
       </c>
-      <c r="W1" s="23"/>
+      <c r="W1" s="27"/>
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" s="13" t="s">
@@ -886,10 +886,10 @@
       <c r="H2" s="2">
         <v>1</v>
       </c>
-      <c r="J2" s="25" t="s">
+      <c r="J2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="K2" s="26"/>
+      <c r="K2" s="24"/>
       <c r="L2" s="2">
         <v>1</v>
       </c>
@@ -899,10 +899,10 @@
       <c r="O2" s="2">
         <v>1</v>
       </c>
-      <c r="Q2" s="25" t="s">
+      <c r="Q2" s="23" t="s">
         <v>0</v>
       </c>
-      <c r="R2" s="26"/>
+      <c r="R2" s="24"/>
       <c r="S2" s="6">
         <v>2</v>
       </c>
@@ -979,10 +979,10 @@
       <c r="H4" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="J4" s="25" t="s">
+      <c r="J4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="K4" s="26"/>
+      <c r="K4" s="24"/>
       <c r="L4" s="18" t="s">
         <v>75</v>
       </c>
@@ -992,10 +992,10 @@
       <c r="O4" s="2">
         <v>1</v>
       </c>
-      <c r="Q4" s="25" t="s">
+      <c r="Q4" s="23" t="s">
         <v>17</v>
       </c>
-      <c r="R4" s="26"/>
+      <c r="R4" s="24"/>
       <c r="S4" s="18" t="s">
         <v>75</v>
       </c>
@@ -1022,11 +1022,11 @@
       <c r="F5" s="19"/>
       <c r="G5" s="19"/>
       <c r="H5" s="19"/>
-      <c r="J5" s="27" t="s">
+      <c r="J5" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="K5" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="K5" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="L5" s="18" t="s">
         <v>76</v>
@@ -1038,11 +1038,11 @@
       <c r="O5" s="3" t="s">
         <v>16</v>
       </c>
-      <c r="Q5" s="27" t="s">
+      <c r="Q5" s="25" t="s">
+        <v>85</v>
+      </c>
+      <c r="R5" s="6" t="s">
         <v>83</v>
-      </c>
-      <c r="R5" s="6" t="s">
-        <v>86</v>
       </c>
       <c r="S5" s="18" t="s">
         <v>76</v>
@@ -1071,9 +1071,9 @@
       <c r="F6" s="21"/>
       <c r="G6" s="21"/>
       <c r="H6" s="21"/>
-      <c r="J6" s="28"/>
+      <c r="J6" s="26"/>
       <c r="K6" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L6" s="6" t="s">
         <v>79</v>
@@ -1084,9 +1084,9 @@
       <c r="O6" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="Q6" s="28"/>
+      <c r="Q6" s="26"/>
       <c r="R6" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="S6" s="6" t="s">
         <v>79</v>
@@ -1105,11 +1105,11 @@
       <c r="B7" s="22" t="s">
         <v>13</v>
       </c>
-      <c r="J7" s="27" t="s">
-        <v>84</v>
+      <c r="J7" s="25" t="s">
+        <v>86</v>
       </c>
       <c r="K7" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L7" s="18" t="s">
         <v>77</v>
@@ -1120,11 +1120,11 @@
       <c r="O7" s="4">
         <v>43263</v>
       </c>
-      <c r="Q7" s="27" t="s">
-        <v>84</v>
+      <c r="Q7" s="25" t="s">
+        <v>86</v>
       </c>
       <c r="R7" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="S7" s="18" t="s">
         <v>77</v>
@@ -1143,9 +1143,9 @@
       <c r="B8" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J8" s="28"/>
+      <c r="J8" s="26"/>
       <c r="K8" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L8" s="6" t="s">
         <v>80</v>
@@ -1156,9 +1156,9 @@
       <c r="O8" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="Q8" s="28"/>
+      <c r="Q8" s="26"/>
       <c r="R8" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="S8" s="6" t="s">
         <v>82</v>
@@ -1177,20 +1177,20 @@
       <c r="B9" s="2" t="s">
         <v>16</v>
       </c>
-      <c r="J9" s="27" t="s">
-        <v>85</v>
+      <c r="J9" s="25" t="s">
+        <v>87</v>
       </c>
       <c r="K9" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="L9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="Q9" s="27" t="s">
-        <v>85</v>
+      <c r="Q9" s="25" t="s">
+        <v>87</v>
       </c>
       <c r="R9" s="6" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="S9" s="18" t="s">
         <v>78</v>
@@ -1209,16 +1209,16 @@
       <c r="B10" s="4">
         <v>43221</v>
       </c>
-      <c r="J10" s="28"/>
+      <c r="J10" s="26"/>
       <c r="K10" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="L10" s="6" t="s">
         <v>81</v>
       </c>
-      <c r="Q10" s="28"/>
+      <c r="Q10" s="26"/>
       <c r="R10" s="6" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="S10" s="6" t="s">
         <v>81</v>
@@ -1270,16 +1270,6 @@
     </row>
   </sheetData>
   <mergeCells count="17">
-    <mergeCell ref="J2:K2"/>
-    <mergeCell ref="J4:K4"/>
-    <mergeCell ref="J5:J6"/>
-    <mergeCell ref="J7:J8"/>
-    <mergeCell ref="J9:J10"/>
-    <mergeCell ref="Q2:R2"/>
-    <mergeCell ref="Q4:R4"/>
-    <mergeCell ref="Q5:Q6"/>
-    <mergeCell ref="Q7:Q8"/>
-    <mergeCell ref="Q9:Q10"/>
     <mergeCell ref="V1:W1"/>
     <mergeCell ref="A1:B1"/>
     <mergeCell ref="D1:E1"/>
@@ -1287,6 +1277,16 @@
     <mergeCell ref="Q1:S1"/>
     <mergeCell ref="G1:H1"/>
     <mergeCell ref="N1:O1"/>
+    <mergeCell ref="Q2:R2"/>
+    <mergeCell ref="Q4:R4"/>
+    <mergeCell ref="Q5:Q6"/>
+    <mergeCell ref="Q7:Q8"/>
+    <mergeCell ref="Q9:Q10"/>
+    <mergeCell ref="J2:K2"/>
+    <mergeCell ref="J4:K4"/>
+    <mergeCell ref="J5:J6"/>
+    <mergeCell ref="J7:J8"/>
+    <mergeCell ref="J9:J10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -1307,18 +1307,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="E1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="23"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1486,14 +1486,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="23"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1630,14 +1630,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="23"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1774,14 +1774,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="23"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -1916,10 +1916,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>44</v>
       </c>
-      <c r="B1" s="23"/>
+      <c r="B1" s="27"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2025,18 +2025,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>25</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="E1" s="23"/>
-      <c r="G1" s="23" t="s">
+      <c r="E1" s="27"/>
+      <c r="G1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="23"/>
+      <c r="H1" s="27"/>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2204,14 +2204,14 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>28</v>
       </c>
-      <c r="B1" s="23"/>
-      <c r="D1" s="23" t="s">
+      <c r="B1" s="27"/>
+      <c r="D1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="E1" s="23"/>
+      <c r="E1" s="27"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">
@@ -2346,10 +2346,10 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.25">
-      <c r="A1" s="23" t="s">
+      <c r="A1" s="27" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="23"/>
+      <c r="B1" s="27"/>
     </row>
     <row r="2" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A2" s="2" t="s">

</xml_diff>